<commit_message>
Add future offline marketing responsibilities
</commit_message>
<xml_diff>
--- a/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
+++ b/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
@@ -1155,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.75" defaultRowHeight="14.25" outlineLevelRow="3"/>
   <cols>
     <col width="5.83333333333333" customWidth="1" style="2" min="1" max="2"/>
@@ -1399,7 +1399,7 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="G7" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -2195,11 +2195,11 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>营销知识库与工作智能体建设</t>
+          <t>线上线下营销Skill复用与场景落地（未来职责）</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -2213,12 +2213,12 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>将产品库、达人看板、活动日历、数据复盘和Agency评估中的稳定规则沉淀为共享总台、标准模板和可复用Skill。维护跨工作台的交接规则、任务状态和资料入口。</t>
+          <t>盘点线上投放、内容运营与线下市场执行中可复用的规则、模板和数据字段，沉淀为共享Skill并明确适用场景、输入输出和人工确认点。维护跨工作台的交接规则、任务状态和资料入口。</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>减少重复搭建和信息孤岛，让日常营销工作可以复用、协作和持续优化。以可复用Skill数量、资料可找到率、交接完整性和人工重复工作减少情况评估。</t>
+          <t>让线上和线下团队复用同一套方法与证据，减少重复搭建和口径断裂。以Skill复用次数、场景覆盖率、交接完整性和人工重复工作减少情况评估。</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -2275,11 +2275,11 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>海外市场与竞品内容调研支持</t>
+          <t>线下市场竞品情报与机会研判（未来职责）</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>根据新品、活动或市场问题收集竞品内容、价格、促销与社媒案例，按产品、国家和平台归类，提炼可验证的机会与风险。将结论输入产品资料库、Brief或活动方案。</t>
+          <t>根据国家、门店、渠道或新品问题收集线下竞品的产品陈列、价格、促销、渠道覆盖和消费者反馈，按市场与产品归类并标注证据来源。将结论输入产品重要级判断、渠道策略、Brief和活动方案。</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>为选品、内容方向和市场决策提供可追溯证据，减少仅凭经验判断。以调研交付及时性、证据可追溯性和结论被采纳情况评估。</t>
+          <t>为线下市场的产品优先级、内容表达和资源投放提供可追溯证据，减少仅凭经验判断。以情报更新时效、证据可追溯性和结论被采纳情况评估。</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -2322,6 +2322,86 @@
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="102" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>海外营销相关部门（待确认）</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>海外KOL/整合营销岗位（待确认）</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>添可智能科技有限公司（待确认）</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>线下渠道策略、预算建议与线上引流转化链路优化（未来职责）</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>按订单/项目/批次/对象发生</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>上级或会议安排、协作中心/系统/智能体触发、自己发现问题、现场/客户/门店/供应商触发</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>结合线下渠道覆盖、竞品情报、产品重要级、活动数据和线上内容表现，梳理投放资源向市场、渠道和产品分配的建议。设计并跟踪线上内容或投放引流至线下门店的转化链路，将渠道策略、产品优先级和本地行动要求反馈到Brief及活动计划。</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>让投放分配、线下渠道目标和内容要求基于同一条转化链路协同，而不是各自独立执行。以重点产品/渠道覆盖率、线上到店线索可追踪率、资源建议采纳情况和转化改善趋势评估。</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>人和硅基共同完成</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>发起和协作、执行、审核或确认、规则维护、智能体建设及调优</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认、涉及沟通关系或体验</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>可由人手动创建希望未来自动触发</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
         </is>

</xml_diff>

<commit_message>
Make future responsibilities MECE
</commit_message>
<xml_diff>
--- a/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
+++ b/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
@@ -1155,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.75" defaultRowHeight="14.25" outlineLevelRow="3"/>
   <cols>
     <col width="5.83333333333333" customWidth="1" style="2" min="1" max="2"/>
@@ -2195,11 +2195,11 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>线上线下营销Skill复用与场景落地（未来职责）</t>
+          <t>营销流程标准化与线上线下Skill运营（未来职责）</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -2275,11 +2275,11 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>线下市场竞品情报与机会研判（未来职责）</t>
+          <t>线下市场竞品情报（未来职责）</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>根据国家、门店、渠道或新品问题收集线下竞品的产品陈列、价格、促销、渠道覆盖和消费者反馈，按市场与产品归类并标注证据来源。将结论输入产品重要级判断、渠道策略、Brief和活动方案。</t>
+          <t>根据国家和产品问题收集线下竞品的产品、价格、促销、陈列和消费者反馈，按市场与产品归类并标注证据来源。输出竞品变化、差异点和待验证假设，不负责渠道选择或预算分配。</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>为线下市场的产品优先级、内容表达和资源投放提供可追溯证据，减少仅凭经验判断。以情报更新时效、证据可追溯性和结论被采纳情况评估。</t>
+          <t>为产品和市场判断提供可追溯的竞争证据，减少仅凭经验判断。以情报更新时效、证据可追溯性和结论被采纳情况评估。</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -2355,53 +2355,133 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>线下渠道策略、预算建议与线上引流转化链路优化（未来职责）</t>
+          <t>线下渠道与终端机会地图（未来职责）</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
+          <t>每月</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>固定时间、上级或会议安排、现场/客户/门店/供应商触发、自己发现问题</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>汇总市场内渠道类型、门店/终端覆盖、经销与零售伙伴、陈列与促销资源、可获得数据和执行限制，形成按国家和渠道的机会地图。输出渠道现状、机会缺口与可测试场景，不负责竞品研究或最终预算审批。</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>让线下市场资源、终端机会和数据缺口被统一看见，为后续优先级和转化策略提供基础。以渠道资料完整率、重点终端覆盖率、机会地图更新及时性评估。</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>人和硅基共同完成</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>执行、发起和协作、审核或确认、规则维护</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>输入数据或系统接口还不完整、必须到现场或接触实物、涉及沟通关系或体验</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>可由人手动创建希望未来自动触发</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="102" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>海外营销相关部门（待确认）</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>海外KOL/整合营销岗位（待确认）</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>添可智能科技有限公司（待确认）</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>产品优先级、资源投放与线上引流到线下转化策略（未来职责）</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
           <t>按订单/项目/批次/对象发生</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>上级或会议安排、协作中心/系统/智能体触发、自己发现问题、现场/客户/门店/供应商触发</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>结合线下渠道覆盖、竞品情报、产品重要级、活动数据和线上内容表现，梳理投放资源向市场、渠道和产品分配的建议。设计并跟踪线上内容或投放引流至线下门店的转化链路，将渠道策略、产品优先级和本地行动要求反馈到Brief及活动计划。</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>让投放分配、线下渠道目标和内容要求基于同一条转化链路协同，而不是各自独立执行。以重点产品/渠道覆盖率、线上到店线索可追踪率、资源建议采纳情况和转化改善趋势评估。</t>
-        </is>
-      </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>上级或会议安排、协作中心/系统/智能体触发、上游岗位交付、自己发现问题</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>基于产品资料、竞品情报、渠道机会地图、活动表现和成本数据，形成各市场的产品重要级、资源投放和预算建议。设计线上内容或投放引流至线下门店的转化链路、埋点和验证方式，并将已确认的优先级与本地行动要求作为 Brief 的输入。</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>把市场证据转化为可执行的资源选择和可验证的线上到线下增长方案。以重点产品/渠道覆盖率、资源建议采纳情况、线上到店线索可追踪率和转化改善趋势评估。</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>人和硅基共同完成</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>发起和协作、执行、审核或确认、规则维护、智能体建设及调优</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认、涉及沟通关系或体验</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>可由人手动创建希望未来自动触发</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="P17" s="3" t="inlineStr">
         <is>
           <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
         </is>

</xml_diff>

<commit_message>
Align role draft to campaign operating chain
</commit_message>
<xml_diff>
--- a/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
+++ b/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
@@ -1315,11 +1315,11 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>海外产品资料库维护与市场适配</t>
+          <t>海外产品与市场资料库维护</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
@@ -1333,12 +1333,12 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>汇总产品规格、卖点、SKU、价格和物料状态，按国家与市场类型标准化，并标记缺失或冲突信息。输出可检索的产品底库，供KOL选品、Brief和活动方案使用。</t>
+          <t>汇总产品规格、SKU、卖点、价格、物料状态和市场适配信息，按国家和产品标准化并标记缺失或冲突。输出可检索的产品与市场资料库，供活动规划和内容策略调用。</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>形成按产品和市场可追溯的统一事实底座，减少重复向产品或当地团队确认。以资料完整性、冲突项闭环率和更新及时性评估。</t>
+          <t>形成可追溯的产品事实底座，减少重复向产品或当地团队确认。以资料完整性、冲突项闭环率和更新及时性评估。</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -1395,30 +1395,30 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>海外KOL/达人信息库整理与更新</t>
+          <t>营销流程标准化与线上线下Skill运营（未来职责）</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>每周</t>
+          <t>每月</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>固定时间、上游岗位交付、自己发现问题</t>
+          <t>自己发现问题、协作中心/系统/智能体触发、上级或会议安排</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>收集法国、意大利、德国等市场的达人资料，统一账号、平台、品类、受众、报价、内容表现和合作状态字段。清洗重复和缺失信息后更新固定看板与达人底库。</t>
+          <t>将活动规划、达人执行、数据复盘和线下市场执行中稳定的规则、模板与字段沉淀为共享Skill，定义输入、输出、适用场景和人工确认点。维护跨工作台的交接规则与资料入口。</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>让达人筛选和历史合作查询有统一入口，减少人工翻找与重复录入。以可用达人数量、字段完整率、重复率和更新时效评估。</t>
+          <t>让线上和线下团队复用同一套方法，减少重复搭建和口径断裂。以Skill复用次数、场景覆盖率和交接完整性评估。</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1428,12 +1428,12 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>执行、规则维护、智能体建设及调优</t>
+          <t>发起和协作、规则维护、智能体建设及调优、最终负责</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及沟通关系或体验</t>
+          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -1475,11 +1475,11 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>活动达人筛选与匹配</t>
+          <t>活动预算拆解与资源分配建议</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -1493,12 +1493,12 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>根据产品、国家、预算、平台、受众、内容风格和历史表现筛选候选达人，形成分层名单及推荐理由。将候选名单交付给项目负责人或当地团队确认。</t>
+          <t>基于活动目标、产品重要级、市场与渠道现状、历史效果和资源限制，拆解达人、内容、投放与线下执行预算，形成按市场、产品和渠道的资源分配建议。将建议提交项目负责人或业务负责人确认。</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>提高达人与活动目标、产品卖点和市场需求的匹配度，降低无效沟通。以名单交付及时性、入选率、合作转化和后续内容表现评估。</t>
+          <t>使资源投向与活动优先级一致，避免预算仅按经验平均分配。以预算拆解完整性、资源建议采纳情况和重点资源覆盖率评估。</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>执行、发起和协作、审核或确认、规则维护</t>
+          <t>执行、发起和协作、审核或确认</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>判断规则还没有沉淀清楚、涉及沟通关系或体验、涉及责任风险或最终确认</t>
+          <t>判断规则还没有沉淀清楚、涉及责任风险或最终确认、输入数据或系统接口还不完整</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
@@ -1555,11 +1555,11 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>KOL合作邀约与进度管理</t>
+          <t>活动目标制定与线上引流到线下衡量框架设计</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -1568,42 +1568,42 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>上级或会议安排、上游岗位交付、现场/客户/门店/供应商触发</t>
+          <t>上级或会议安排、协作中心/系统/智能体触发、上游岗位交付</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>基于确认名单发起邀约，沟通合作条件、产品寄送、档期和交付要求，持续更新回复、签约、寄样、发布和异常状态。向项目负责人同步关键风险与下一步动作。</t>
+          <t>将业务目标拆解为市场、产品、内容、达人、投放和线下转化目标，明确线上内容或投放引流至线下门店的路径、可获得数据、埋点与验证方式。输出活动目标表和衡量口径。</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>保障合作链路可追踪并减少遗漏，及时处理档期、报价和交付异常。以有效回复率、合作确认率、节点准时率和异常闭环率评估。</t>
+          <t>让活动从开始就具备可追踪的成功标准，并识别线上到线下链路的数据缺口。以目标清晰度、口径一致性和关键转化指标可追踪率评估。</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>主要由人完成</t>
+          <t>人和硅基共同完成</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>执行、发起和协作、例外处理</t>
+          <t>发起和协作、执行、审核或确认、规则维护</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>涉及沟通关系或体验、涉及责任风险或最终确认、输入数据或系统接口还不完整</t>
+          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>已进入一部分但不完整</t>
+          <t>可由人手动创建希望未来自动触发</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>协作中心/任务中心、飞书文档/表格、飞书群或私聊、Excel本地文件</t>
+          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
         </is>
       </c>
     </row>
@@ -1635,11 +1635,11 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>海外KOL产品Brief与内容要求制定</t>
+          <t>活动内容策略与KOL Brief规划</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -1648,17 +1648,17 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>上级或会议安排、上游岗位交付、协作中心/系统/智能体触发</t>
+          <t>上级或会议安排、上游岗位交付、自己发现问题</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>结合产品资料、市场洞察、活动目标和达人内容特点，编写英文产品Brief、卖点、脚本方向、交付物、禁忌和发布要求。经产品、品牌或项目负责人确认后交付达人及Agency。</t>
+          <t>围绕活动目标完成竞品内容分析、线下下店/到店量及终端反馈分析，确定产品卖点、内容角度、平台表达和本地行动要求。将已确认策略转化为英文KOL Brief、脚本方向、交付物、禁忌和发布要求。</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>统一内容口径并把产品卖点转化为可执行的创作要求，降低返工和表达偏差。以Brief确认时效、内容一次通过率和关键卖点覆盖率评估。</t>
+          <t>使竞品与线下市场证据真正影响内容表达和Brief，而不是停留在调研报告中。以Brief确认时效、关键卖点覆盖率、内容一次通过率和策略被采纳情况评估。</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -1715,11 +1715,11 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>KOL内容审核、修改与发布追踪</t>
+          <t>活动达人策略制定</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -1728,17 +1728,17 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>上游岗位交付、协作中心/系统/智能体触发、现场/客户/门店/供应商触发</t>
+          <t>上级或会议安排、协作中心/系统/智能体触发、上游岗位交付</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>审核达人脚本、素材和成片是否覆盖产品卖点、符合品牌表达及平台规范，整理修改意见并跟进定稿与发布时间。将链接、交付状态和复用素材沉淀到项目记录。</t>
+          <t>根据活动目标、预算、内容策略、市场和产品优先级，确定达人平台、圈层、数量、分层、内容角色和合作节奏。输出达人策略及筛选标准，作为达人筛选和建联的统一依据。</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>保障内容合规、信息准确和按计划上线，并形成后续投放和复盘可用素材。以准时发布率、修改轮次、合规问题数和可复用素材数量评估。</t>
+          <t>让达人资源与内容和投放目标匹配，避免先找达人再补策略。以策略交付及时性、筛选标准完整性、合作确认率和后续内容表现评估。</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1748,17 +1748,17 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>执行、审核或确认、例外处理</t>
+          <t>执行、发起和协作、审核或确认、规则维护</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>涉及责任风险或最终确认、涉及沟通关系或体验、判断规则还没有沉淀清楚</t>
+          <t>判断规则还没有沉淀清楚、涉及沟通关系或体验、涉及责任风险或最终确认</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>已进入一部分但不完整</t>
+          <t>可由人手动创建希望未来自动触发</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>跨市场整合营销活动项目推进</t>
+          <t>投放节点与素材供给规划</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
@@ -1808,32 +1808,32 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>上级或会议安排、协作中心/系统/智能体触发、上游岗位交付</t>
+          <t>上级或会议安排、固定时间、上游岗位交付</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>围绕法国、意大利、德国等市场的活动目标，协调产品、KOL、Agency、当地团队与投放节点，拆解交付物、排期、预算和风险。维护活动总表并推动关键节点按时完成。</t>
+          <t>依据活动排期、达人内容交付、产品与渠道节奏，规划Meta等投放的上线节点、素材需求、责任人和备选方案。维护投放日历并同步素材缺口和节点变化。</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>让多方工作围绕同一目标和时间表推进，避免资源与信息脱节。以里程碑准时率、关键交付完成率、预算及风险问题闭环情况评估。</t>
+          <t>让投放节奏与内容供给、线下活动节点一致，降低漏投、错配和临近节点返工。以节点覆盖率、素材按时到位率和日历更新及时性评估。</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>主要由人完成</t>
+          <t>人和硅基共同完成</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>发起和协作、例外处理、最终负责</t>
+          <t>执行、发起和协作、规则维护</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>涉及沟通关系或体验、涉及责任风险或最终确认、输入数据或系统接口还不完整</t>
+          <t>输入数据或系统接口还不完整、涉及沟通关系或体验、涉及责任风险或最终确认</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1875,11 +1875,11 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Meta投放日历与素材节点统筹</t>
+          <t>海外KOL/达人信息库整理与更新</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -1888,17 +1888,17 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>固定时间、上级或会议安排、上游岗位交付</t>
+          <t>固定时间、上游岗位交付、自己发现问题</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>整合各市场活动、KOL内容、产品和投放计划，维护Meta投放日历中的上线日期、素材状态、责任人和待确认事项。向相关团队同步素材缺口和节点变化。</t>
+          <t>收集法国、意大利、德国等市场的达人资料，统一账号、平台、品类、受众、报价、内容表现和合作状态字段。清洗重复和缺失信息后更新固定看板与达人底库。</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>使投放安排与内容供给可视化，降低漏投、素材错配和临近节点返工。以节点覆盖率、素材按时到位率和日历更新及时性评估。</t>
+          <t>让筛选和历史合作查询有统一入口，减少人工翻找与重复录入。以字段完整率、重复率、可用达人数量和更新时效评估。</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1908,12 +1908,12 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>执行、发起和协作、规则维护</t>
+          <t>执行、规则维护、智能体建设及调优</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>输入数据或系统接口还不完整、涉及沟通关系或体验、涉及责任风险或最终确认</t>
+          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及沟通关系或体验</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>协作中心/任务中心、飞书文档/表格、Excel本地文件</t>
+          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
         </is>
       </c>
     </row>
@@ -1955,30 +1955,30 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>活动投放素材与数据源整理校验</t>
+          <t>活动达人筛选与匹配</t>
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>每周</t>
+          <t>按订单/项目/批次/对象发生</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>固定时间、上游岗位交付、协作中心/系统/智能体触发、自己发现问题</t>
+          <t>上游岗位交付、协作中心/系统/智能体触发、上级或会议安排</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>收集Meta、社媒平台、Agency和达人侧的素材与原始数据，统一命名、市场、产品、平台和时间口径，并核对缺失、重复及异常值。输出可用于分析和复盘的清洁数据集。</t>
+          <t>依据已确认的达人策略和筛选标准，从达人库筛选候选人，核对受众、内容风格、报价、档期和历史表现，形成分层名单及推荐理由。将候选名单交付项目负责人或当地团队确认。</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>提高数据可用性和分析结论可信度，避免基于错误口径做决策。以数据完整率、异常发现与闭环率、口径一致性和可追溯性评估。</t>
+          <t>提高达人与活动目标、产品卖点和市场需求的匹配度，降低无效沟通。以名单交付及时性、入选率、合作转化和后续内容表现评估。</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1988,17 +1988,17 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>执行、审核或确认、规则维护、智能体建设及调优</t>
+          <t>执行、发起和协作、审核或确认、规则维护</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认</t>
+          <t>判断规则还没有沉淀清楚、涉及沟通关系或体验、涉及责任风险或最终确认</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>已进入一部分但不完整</t>
+          <t>可由人手动创建希望未来自动触发</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -2035,55 +2035,55 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>活动效果诊断与复盘行动制定</t>
+          <t>KOL建联与合作进度管理</t>
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>每月</t>
+          <t>按订单/项目/批次/对象发生</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>固定时间、上级或会议安排、协作中心/系统/智能体触发</t>
+          <t>上游岗位交付、现场/客户/门店/供应商触发、上级或会议安排</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>基于清洗后的活动和投放数据，按市场、产品、达人、内容和渠道分析表现，识别有效做法、问题与证据缺口。输出复盘结论及保留、停止、测试或修复的下一步行动。</t>
+          <t>基于确认名单发起邀约，沟通合作条件、产品寄送、档期和交付要求，持续更新回复、签约、寄样、发布和异常状态。向项目负责人同步关键风险与下一步动作。</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>把活动结果沉淀为下一轮可执行的优化动作，而非只汇报数据。以复盘交付及时性、行动项闭环率和后续测试结果评估。</t>
+          <t>保障合作链路可追踪并及时处理档期、报价和交付异常。以有效回复率、合作确认率、节点准时率和异常闭环率评估。</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>人和硅基共同完成</t>
+          <t>主要由人完成</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>执行、审核或确认、发起和协作、智能体建设及调优</t>
+          <t>执行、发起和协作、例外处理</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>判断规则还没有沉淀清楚、涉及责任风险或最终确认、输入数据或系统接口还不完整</t>
+          <t>涉及沟通关系或体验、涉及责任风险或最终确认、输入数据或系统接口还不完整</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>可由人手动创建希望未来自动触发</t>
+          <t>已进入一部分但不完整</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
+          <t>协作中心/任务中心、飞书文档/表格、飞书群或私聊、Excel本地文件</t>
         </is>
       </c>
     </row>
@@ -2115,30 +2115,30 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>海外Agency报告评估与合作质量管理</t>
+          <t>KOL内容审核、修改与发布追踪</t>
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>每月</t>
+          <t>按订单/项目/批次/对象发生</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>固定时间、上游岗位交付、现场/客户/门店/供应商触发</t>
+          <t>上游岗位交付、协作中心/系统/智能体触发、现场/客户/门店/供应商触发</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>汇总法国、意大利、德国Agency的过程记录、交付物和效果数据，按统一标准检查资料完整性、执行质量、结果价值和问题。形成评估结论、反馈要点及后续合作建议。</t>
+          <t>审核达人脚本、素材和成片是否符合确认后的内容策略、Brief、品牌表达及平台规范，整理修改意见并跟进定稿与发布时间。将链接、交付状态和复用素材沉淀到项目记录。</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>提高外部合作的可比性与验收质量，明确哪些合作方式应保留或调整。以报告完整性、交付准时率、问题闭环率和建议采纳情况评估。</t>
+          <t>保障内容合规、准确并按计划上线，形成可用于投放和复盘的素材资产。以准时发布率、修改轮次、合规问题数和可复用素材数量评估。</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -2148,12 +2148,12 @@
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>执行、审核或确认、例外处理、规则维护</t>
+          <t>执行、审核或确认、例外处理</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>涉及责任风险或最终确认、输入数据或系统接口还不完整、判断规则还没有沉淀清楚</t>
+          <t>涉及责任风险或最终确认、涉及沟通关系或体验、判断规则还没有沉淀清楚</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
@@ -2195,30 +2195,30 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>营销流程标准化与线上线下Skill运营（未来职责）</t>
+          <t>活动进展周报与海外上游团队同步</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>每月</t>
+          <t>每周</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>自己发现问题、协作中心/系统/智能体触发、上级或会议安排</t>
+          <t>固定时间、上游岗位交付、自己发现问题</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>盘点线上投放、内容运营与线下市场执行中可复用的规则、模板和数据字段，沉淀为共享Skill并明确适用场景、输入输出和人工确认点。维护跨工作台的交接规则、任务状态和资料入口。</t>
+          <t>汇总活动预算、达人、内容、投放和线下转化的本周进展、已完成事项、风险和需决策事项，向海外上游团队及项目相关方输出周报。更新活动总表和下一周行动清单。</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>让线上和线下团队复用同一套方法与证据，减少重复搭建和口径断裂。以Skill复用次数、场景覆盖率、交接完整性和人工重复工作减少情况评估。</t>
+          <t>让海外上游团队及时掌握真实进度和风险，减少重复追问与信息滞后。以周报准时率、关键信息完整性和风险闭环率评估。</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -2228,12 +2228,12 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>发起和协作、规则维护、智能体建设及调优、最终负责</t>
+          <t>执行、发起和协作、例外处理</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认</t>
+          <t>涉及沟通关系或体验、输入数据或系统接口还不完整、涉及责任风险或最终确认</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
+          <t>协作中心/任务中心、飞书文档/表格、飞书群或私聊、Excel本地文件</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>线下市场竞品情报（未来职责）</t>
+          <t>活动素材与数据源整理校验</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
@@ -2283,22 +2283,22 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>按订单/项目/批次/对象发生</t>
+          <t>每周</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>上级或会议安排、自己发现问题、协作中心/系统/智能体触发</t>
+          <t>固定时间、上游岗位交付、协作中心/系统/智能体触发、自己发现问题</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>根据国家和产品问题收集线下竞品的产品、价格、促销、陈列和消费者反馈，按市场与产品归类并标注证据来源。输出竞品变化、差异点和待验证假设，不负责渠道选择或预算分配。</t>
+          <t>收集Meta、社媒平台、Agency、达人和线下渠道侧的素材与原始数据，统一命名、市场、产品、平台和时间口径，并核对缺失、重复及异常值。输出可用于衡量和复盘的清洁数据集。</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>为产品和市场判断提供可追溯的竞争证据，减少仅凭经验判断。以情报更新时效、证据可追溯性和结论被采纳情况评估。</t>
+          <t>提高数据可用性和分析结论可信度，避免基于错误口径做决策。以数据完整率、异常闭环率、口径一致性和可追溯性评估。</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>执行、发起和协作、审核或确认、智能体建设及调优</t>
+          <t>执行、审核或确认、规则维护、智能体建设及调优</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>可由人手动创建希望未来自动触发</t>
+          <t>已进入一部分但不完整</t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>线下渠道与终端机会地图（未来职责）</t>
+          <t>活动效果复盘与下一轮行动制定</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
@@ -2368,17 +2368,17 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>固定时间、上级或会议安排、现场/客户/门店/供应商触发、自己发现问题</t>
+          <t>固定时间、上级或会议安排、协作中心/系统/智能体触发</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>汇总市场内渠道类型、门店/终端覆盖、经销与零售伙伴、陈列与促销资源、可获得数据和执行限制，形成按国家和渠道的机会地图。输出渠道现状、机会缺口与可测试场景，不负责竞品研究或最终预算审批。</t>
+          <t>基于确认的目标和清洗后的数据，按市场、产品、达人、内容、投放和线上到线下转化链路分析表现，识别有效做法、问题与证据缺口。输出保留、停止、测试或修复的下一轮行动。</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>让线下市场资源、终端机会和数据缺口被统一看见，为后续优先级和转化策略提供基础。以渠道资料完整率、重点终端覆盖率、机会地图更新及时性评估。</t>
+          <t>把活动结果沉淀为可执行的优化动作，而非只汇报数据。以复盘交付及时性、行动项闭环率和后续测试结果评估。</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -2388,12 +2388,12 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>执行、发起和协作、审核或确认、规则维护</t>
+          <t>执行、审核或确认、发起和协作、智能体建设及调优</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>输入数据或系统接口还不完整、必须到现场或接触实物、涉及沟通关系或体验</t>
+          <t>判断规则还没有沉淀清楚、涉及责任风险或最终确认、输入数据或系统接口还不完整</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
@@ -2435,30 +2435,30 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>产品优先级、资源投放与线上引流到线下转化策略（未来职责）</t>
+          <t>海外Agency交付评估与合作质量管理</t>
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>按订单/项目/批次/对象发生</t>
+          <t>每月</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>上级或会议安排、协作中心/系统/智能体触发、上游岗位交付、自己发现问题</t>
+          <t>固定时间、上游岗位交付、现场/客户/门店/供应商触发</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>基于产品资料、竞品情报、渠道机会地图、活动表现和成本数据，形成各市场的产品重要级、资源投放和预算建议。设计线上内容或投放引流至线下门店的转化链路、埋点和验证方式，并将已确认的优先级与本地行动要求作为 Brief 的输入。</t>
+          <t>汇总Agency的过程记录、交付物和效果数据，按统一标准检查资料完整性、执行质量、结果价值和问题。形成评估结论、反馈要点及后续合作建议。</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>把市场证据转化为可执行的资源选择和可验证的线上到线下增长方案。以重点产品/渠道覆盖率、资源建议采纳情况、线上到店线索可追踪率和转化改善趋势评估。</t>
+          <t>提高外部合作的可比性与验收质量，明确哪些合作方式应保留或调整。以报告完整性、交付准时率、问题闭环率和建议采纳情况评估。</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -2468,17 +2468,17 @@
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>发起和协作、执行、审核或确认、规则维护、智能体建设及调优</t>
+          <t>执行、审核或确认、例外处理、规则维护</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认、涉及沟通关系或体验</t>
+          <t>涉及责任风险或最终确认、输入数据或系统接口还不完整、判断规则还没有沉淀清楚</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>可由人手动创建希望未来自动触发</t>
+          <t>已进入一部分但不完整</t>
         </is>
       </c>
       <c r="P17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add special projects and conversion capability
</commit_message>
<xml_diff>
--- a/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
+++ b/projects/job-role-research/2026-09-24/岗位素材调研_海外营销工作初稿.xlsx
@@ -1155,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.75" defaultRowHeight="14.25" outlineLevelRow="3"/>
   <cols>
     <col width="5.83333333333333" customWidth="1" style="2" min="1" max="2"/>
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="G3" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
@@ -1399,7 +1399,7 @@
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -1555,11 +1555,11 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>活动目标制定与线上引流到线下衡量框架设计</t>
+          <t>活动目标制定与转化衡量框架配置</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -1573,12 +1573,12 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>将业务目标拆解为市场、产品、内容、达人、投放和线下转化目标，明确线上内容或投放引流至线下门店的路径、可获得数据、埋点与验证方式。输出活动目标表和衡量口径。</t>
+          <t>基于既定转化机制，将单场活动目标拆解为市场、产品、内容、达人、投放和线下转化目标，配置可获得数据、埋点与衡量口径。输出活动目标表和衡量框架，不负责跨活动转化机制建设。</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>让活动从开始就具备可追踪的成功标准，并识别线上到线下链路的数据缺口。以目标清晰度、口径一致性和关键转化指标可追踪率评估。</t>
+          <t>让单场活动从开始就具备可追踪的成功标准，并暴露数据缺口。以目标清晰度、口径一致性和关键转化指标可追踪率评估。</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="G7" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="G8" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -2482,6 +2482,166 @@
         </is>
       </c>
       <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="102" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>海外营销相关部门（待确认）</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>海外KOL/整合营销岗位（待确认）</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>添可智能科技有限公司（待确认）</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>特殊整合营销项目方案与跨方统筹（如法国）</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>按订单/项目/批次/对象发生</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>上级或会议安排、上游岗位交付、现场/客户/门店/供应商触发</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>针对法国等非标准整合营销项目，整合线上内容、KOL、投放、线下渠道/门店、Agency和当地团队的目标、资源、排期与风险，形成项目方案、总排期和决策清单。推动关键决策与跨方交付按计划完成。</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>让复杂整合项目以一个统一方案和关键节点推进，避免各团队各自执行但无法形成合力。以方案确认及时性、关键里程碑准时率、跨方问题闭环率和项目目标达成情况评估。</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>主要由人完成</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>发起和协作、审核或确认、例外处理、最终负责</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>涉及沟通关系或体验、涉及责任风险或最终确认、必须到现场或接触实物、输入数据或系统接口还不完整</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>可由人手动创建希望未来自动触发</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>协作中心/任务中心、飞书文档/表格、飞书群或私聊、Excel本地文件</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="102" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>待本人确认</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>海外营销相关部门（待确认）</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>海外KOL/整合营销岗位（待确认）</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>添可智能科技有限公司（待确认）</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>线上引流到线下转化链路建设与试点（未来职责）</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>按订单/项目/批次/对象发生</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>上级或会议安排、自己发现问题、协作中心/系统/智能体触发</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>跨活动设计线上内容和投放到门店、渠道或销售结果的转化路径，明确数据采集、归因规则、试点场景和验证周期。推动与当地团队、渠道伙伴和数据相关方完成试点，并沉淀可复用的转化机制。</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>持续补齐线上到线下的转化闭环，使后续活动可在既有机制上配置目标和指标。以可追踪转化路径覆盖率、试点完成率、数据可用性和有效机制复用情况评估。</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>人和硅基共同完成</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>发起和协作、执行、审核或确认、规则维护、智能体建设及调优</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>输入数据或系统接口还不完整、判断规则还没有沉淀清楚、涉及责任风险或最终确认、涉及沟通关系或体验</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>可由人手动创建希望未来自动触发</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
         <is>
           <t>协作中心/任务中心、智能体平台/Skill平台、飞书文档/表格、Excel本地文件</t>
         </is>

</xml_diff>